<commit_message>
Currently able to store SLE and CEA data in a .csv file for N-component mixture. The data columns are hardcoded and missing the capability to plot/compare the data.
</commit_message>
<xml_diff>
--- a/combinations.xlsx
+++ b/combinations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5CF6CF9-541E-4F54-A7EF-E06656FCC48F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05071610-905F-4DC0-900D-98FCE6A335EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B8C1824D-4D5B-4C7B-AC69-D3150ED7D660}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B8C1824D-4D5B-4C7B-AC69-D3150ED7D660}"/>
   </bookViews>
   <sheets>
     <sheet name="2 Components" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
     <t>Component 1</t>
   </si>
@@ -432,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7123A7AB-A007-4A53-822D-9E7D5E6D36EC}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -452,6 +452,14 @@
       </c>
       <c r="B2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>